<commit_message>
Update to pass foo tests
</commit_message>
<xml_diff>
--- a/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
+++ b/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
@@ -317,7 +317,7 @@
     <t xml:space="preserve">ts_u16</t>
   </si>
   <si>
-    <t xml:space="preserve">PRESENT</t>
+    <t xml:space="preserve">1</t>
   </si>
   <si>
     <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; ts_u11; 70; 90; 73; 81)</t>
@@ -329,7 +329,7 @@
     <t xml:space="preserve">ts_u17</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED</t>
+    <t xml:space="preserve">0</t>
   </si>
   <si>
     <t xml:space="preserve">=ADD(ts_u3;12)</t>

</xml_diff>

<commit_message>
Remove output check for variables that are states
</commit_message>
<xml_diff>
--- a/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
+++ b/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="121">
   <si>
     <t xml:space="preserve">Dummy Test</t>
   </si>
@@ -518,9 +518,6 @@
     <t xml:space="preserve">ts_y21</t>
   </si>
   <si>
-    <t xml:space="preserve">ts_y22</t>
-  </si>
-  <si>
     <t xml:space="preserve">ts_y23</t>
   </si>
   <si>
@@ -531,12 +528,6 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;56</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y26</t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1064,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BZ64"/>
+  <dimension ref="A1:BZ1048576"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="64.17"/>
@@ -6031,22 +6022,22 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="32" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B60" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="C60" s="39" t="n">
+      <c r="C60" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D60" s="34" t="s">
         <v>94</v>
       </c>
       <c r="E60" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F60" s="35" t="s">
-        <v>70</v>
+        <v>118</v>
+      </c>
+      <c r="F60" s="35" t="n">
+        <v>55</v>
       </c>
       <c r="G60" s="36"/>
       <c r="H60" s="36"/>
@@ -6123,10 +6114,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="32" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B61" s="32" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C61" s="33" t="n">
         <v>0</v>
@@ -6135,7 +6126,7 @@
         <v>94</v>
       </c>
       <c r="E61" s="34" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F61" s="35" t="n">
         <v>55</v>
@@ -6213,212 +6204,11 @@
       <c r="BY61" s="36"/>
       <c r="BZ61" s="36"/>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="B62" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="C62" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="E62" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="F62" s="35" t="n">
-        <v>55</v>
-      </c>
-      <c r="G62" s="36"/>
-      <c r="H62" s="36"/>
-      <c r="I62" s="36"/>
-      <c r="J62" s="36"/>
-      <c r="K62" s="36"/>
-      <c r="L62" s="36"/>
-      <c r="M62" s="36"/>
-      <c r="N62" s="36"/>
-      <c r="O62" s="36"/>
-      <c r="P62" s="36"/>
-      <c r="Q62" s="36"/>
-      <c r="R62" s="36"/>
-      <c r="S62" s="36"/>
-      <c r="T62" s="36"/>
-      <c r="U62" s="37"/>
-      <c r="V62" s="36"/>
-      <c r="W62" s="36"/>
-      <c r="X62" s="36"/>
-      <c r="Y62" s="36"/>
-      <c r="Z62" s="36"/>
-      <c r="AA62" s="36"/>
-      <c r="AB62" s="36"/>
-      <c r="AC62" s="36"/>
-      <c r="AD62" s="36"/>
-      <c r="AE62" s="36"/>
-      <c r="AF62" s="36"/>
-      <c r="AG62" s="36"/>
-      <c r="AH62" s="36"/>
-      <c r="AI62" s="36"/>
-      <c r="AJ62" s="36"/>
-      <c r="AK62" s="36"/>
-      <c r="AL62" s="36"/>
-      <c r="AM62" s="37"/>
-      <c r="AN62" s="36"/>
-      <c r="AO62" s="36"/>
-      <c r="AP62" s="36"/>
-      <c r="AQ62" s="36"/>
-      <c r="AR62" s="36"/>
-      <c r="AS62" s="36"/>
-      <c r="AT62" s="36"/>
-      <c r="AU62" s="36"/>
-      <c r="AV62" s="36"/>
-      <c r="AW62" s="37"/>
-      <c r="AX62" s="36"/>
-      <c r="AY62" s="36"/>
-      <c r="AZ62" s="36"/>
-      <c r="BA62" s="36"/>
-      <c r="BB62" s="36"/>
-      <c r="BC62" s="36"/>
-      <c r="BD62" s="36"/>
-      <c r="BE62" s="36"/>
-      <c r="BF62" s="36"/>
-      <c r="BG62" s="36"/>
-      <c r="BH62" s="36"/>
-      <c r="BI62" s="36"/>
-      <c r="BJ62" s="36"/>
-      <c r="BK62" s="36"/>
-      <c r="BL62" s="36"/>
-      <c r="BM62" s="36"/>
-      <c r="BN62" s="36"/>
-      <c r="BO62" s="36"/>
-      <c r="BP62" s="37"/>
-      <c r="BQ62" s="38"/>
-      <c r="BR62" s="36"/>
-      <c r="BS62" s="36"/>
-      <c r="BT62" s="36"/>
-      <c r="BU62" s="36"/>
-      <c r="BV62" s="36"/>
-      <c r="BW62" s="36"/>
-      <c r="BX62" s="36"/>
-      <c r="BY62" s="36"/>
-      <c r="BZ62" s="36"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="B63" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="C63" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="E63" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="F63" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="G63" s="36"/>
-      <c r="H63" s="36"/>
-      <c r="I63" s="36"/>
-      <c r="J63" s="36"/>
-      <c r="K63" s="36"/>
-      <c r="L63" s="36"/>
-      <c r="M63" s="36"/>
-      <c r="N63" s="36"/>
-      <c r="O63" s="36"/>
-      <c r="P63" s="36"/>
-      <c r="Q63" s="36"/>
-      <c r="R63" s="36"/>
-      <c r="S63" s="36"/>
-      <c r="T63" s="36"/>
-      <c r="U63" s="37"/>
-      <c r="V63" s="36"/>
-      <c r="W63" s="36"/>
-      <c r="X63" s="36"/>
-      <c r="Y63" s="36"/>
-      <c r="Z63" s="36"/>
-      <c r="AA63" s="36"/>
-      <c r="AB63" s="36"/>
-      <c r="AC63" s="36"/>
-      <c r="AD63" s="36"/>
-      <c r="AE63" s="36"/>
-      <c r="AF63" s="36"/>
-      <c r="AG63" s="36"/>
-      <c r="AH63" s="36"/>
-      <c r="AI63" s="36"/>
-      <c r="AJ63" s="36"/>
-      <c r="AK63" s="36"/>
-      <c r="AL63" s="36"/>
-      <c r="AM63" s="37"/>
-      <c r="AN63" s="36"/>
-      <c r="AO63" s="36"/>
-      <c r="AP63" s="36"/>
-      <c r="AQ63" s="36"/>
-      <c r="AR63" s="36"/>
-      <c r="AS63" s="36"/>
-      <c r="AT63" s="36"/>
-      <c r="AU63" s="36"/>
-      <c r="AV63" s="36"/>
-      <c r="AW63" s="37"/>
-      <c r="AX63" s="36"/>
-      <c r="AY63" s="36"/>
-      <c r="AZ63" s="36"/>
-      <c r="BA63" s="36"/>
-      <c r="BB63" s="36"/>
-      <c r="BC63" s="36"/>
-      <c r="BD63" s="36"/>
-      <c r="BE63" s="36"/>
-      <c r="BF63" s="36"/>
-      <c r="BG63" s="36"/>
-      <c r="BH63" s="36"/>
-      <c r="BI63" s="36"/>
-      <c r="BJ63" s="36"/>
-      <c r="BK63" s="36"/>
-      <c r="BL63" s="36"/>
-      <c r="BM63" s="36"/>
-      <c r="BN63" s="36"/>
-      <c r="BO63" s="36"/>
-      <c r="BP63" s="37"/>
-      <c r="BQ63" s="38"/>
-      <c r="BR63" s="36"/>
-      <c r="BS63" s="36"/>
-      <c r="BT63" s="36"/>
-      <c r="BU63" s="36"/>
-      <c r="BV63" s="36"/>
-      <c r="BW63" s="36"/>
-      <c r="BX63" s="36"/>
-      <c r="BY63" s="36"/>
-      <c r="BZ63" s="36"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="32" t="s">
-        <v>78</v>
-      </c>
-      <c r="B64" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="C64" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="E64" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="F64" s="35" t="s">
-        <v>80</v>
-      </c>
-    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <conditionalFormatting sqref="G8:ZY33 G39:ZY63">
+  <conditionalFormatting sqref="G8:ZY33 G39:ZY61">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>#ref!&lt;&gt;G8</formula>
     </cfRule>

</xml_diff>

<commit_message>
Fix for allowing step to continue if expression is false, and add better docs
</commit_message>
<xml_diff>
--- a/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
+++ b/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="130">
   <si>
     <t xml:space="preserve">Dummy Test</t>
   </si>
@@ -203,6 +203,9 @@
     <t xml:space="preserve">7</t>
   </si>
   <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
     <t xml:space="preserve">A</t>
   </si>
   <si>
@@ -449,6 +452,9 @@
     <t xml:space="preserve">ts_y1</t>
   </si>
   <si>
+    <t xml:space="preserve">ts_y11</t>
+  </si>
+  <si>
     <t xml:space="preserve">Variable Value</t>
   </si>
   <si>
@@ -461,7 +467,7 @@
     <t xml:space="preserve">&lt;=71</t>
   </si>
   <si>
-    <t xml:space="preserve">ts_y11</t>
+    <t xml:space="preserve">&gt;=70</t>
   </si>
   <si>
     <t xml:space="preserve">Expected Outputs</t>
@@ -1315,7 +1321,9 @@
       <c r="J6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="K6" s="19"/>
+      <c r="K6" s="18" t="s">
+        <v>4</v>
+      </c>
       <c r="L6" s="19"/>
       <c r="M6" s="19"/>
       <c r="N6" s="19"/>
@@ -1418,7 +1426,9 @@
       <c r="J7" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="26"/>
+      <c r="K7" s="25" t="s">
+        <v>12</v>
+      </c>
       <c r="L7" s="26"/>
       <c r="M7" s="26"/>
       <c r="N7" s="26"/>
@@ -1490,10 +1500,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="32" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="33"/>
       <c r="D8" s="34" t="n">
@@ -1517,7 +1527,9 @@
       <c r="J8" s="35" t="n">
         <v>70</v>
       </c>
-      <c r="K8" s="36"/>
+      <c r="K8" s="35" t="n">
+        <v>70</v>
+      </c>
       <c r="L8" s="36"/>
       <c r="M8" s="36"/>
       <c r="N8" s="36"/>
@@ -1589,10 +1601,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" s="33"/>
       <c r="D9" s="35" t="n">
@@ -1616,7 +1628,9 @@
       <c r="J9" s="35" t="n">
         <v>75</v>
       </c>
-      <c r="K9" s="36"/>
+      <c r="K9" s="35" t="n">
+        <v>75</v>
+      </c>
       <c r="L9" s="36"/>
       <c r="M9" s="36"/>
       <c r="N9" s="36"/>
@@ -1688,10 +1702,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" s="39"/>
       <c r="D10" s="35" t="n">
@@ -1715,7 +1729,9 @@
       <c r="J10" s="35" t="n">
         <v>60</v>
       </c>
-      <c r="K10" s="36"/>
+      <c r="K10" s="35" t="n">
+        <v>60</v>
+      </c>
       <c r="L10" s="36"/>
       <c r="M10" s="36"/>
       <c r="N10" s="36"/>
@@ -1787,10 +1803,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" s="39"/>
       <c r="D11" s="35" t="n">
@@ -1814,7 +1830,9 @@
       <c r="J11" s="35" t="n">
         <v>90</v>
       </c>
-      <c r="K11" s="36"/>
+      <c r="K11" s="35" t="n">
+        <v>90</v>
+      </c>
       <c r="L11" s="36"/>
       <c r="M11" s="36"/>
       <c r="N11" s="36"/>
@@ -1886,10 +1904,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12" s="33"/>
       <c r="D12" s="35" t="n">
@@ -1913,7 +1931,9 @@
       <c r="J12" s="35" t="n">
         <v>1000</v>
       </c>
-      <c r="K12" s="36"/>
+      <c r="K12" s="35" t="n">
+        <v>1000</v>
+      </c>
       <c r="L12" s="36"/>
       <c r="M12" s="36"/>
       <c r="N12" s="36"/>
@@ -1985,17 +2005,17 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C13" s="39"/>
       <c r="D13" s="35" t="n">
         <v>500</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F13" s="35" t="n">
         <v>500</v>
@@ -2012,7 +2032,9 @@
       <c r="J13" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="K13" s="36"/>
+      <c r="K13" s="35" t="n">
+        <v>500</v>
+      </c>
       <c r="L13" s="36"/>
       <c r="M13" s="36"/>
       <c r="N13" s="36"/>
@@ -2084,10 +2106,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" s="39"/>
       <c r="D14" s="35" t="n">
@@ -2111,7 +2133,9 @@
       <c r="J14" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="K14" s="36"/>
+      <c r="K14" s="35" t="n">
+        <v>100</v>
+      </c>
       <c r="L14" s="36"/>
       <c r="M14" s="36"/>
       <c r="N14" s="36"/>
@@ -2183,17 +2207,17 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="35" t="n">
         <v>200</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F15" s="35" t="n">
         <v>200</v>
@@ -2210,7 +2234,9 @@
       <c r="J15" s="35" t="n">
         <v>200</v>
       </c>
-      <c r="K15" s="36"/>
+      <c r="K15" s="35" t="n">
+        <v>200</v>
+      </c>
       <c r="L15" s="36"/>
       <c r="M15" s="36"/>
       <c r="N15" s="36"/>
@@ -2282,17 +2308,17 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="32" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="35" t="n">
         <v>120</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F16" s="35" t="n">
         <v>120</v>
@@ -2309,7 +2335,9 @@
       <c r="J16" s="35" t="n">
         <v>120</v>
       </c>
-      <c r="K16" s="36"/>
+      <c r="K16" s="35" t="n">
+        <v>120</v>
+      </c>
       <c r="L16" s="36"/>
       <c r="M16" s="36"/>
       <c r="N16" s="36"/>
@@ -2381,17 +2409,17 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C17" s="33"/>
       <c r="D17" s="35" t="n">
         <v>20</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F17" s="35" t="n">
         <v>20</v>
@@ -2408,7 +2436,9 @@
       <c r="J17" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="K17" s="36"/>
+      <c r="K17" s="35" t="n">
+        <v>20</v>
+      </c>
       <c r="L17" s="36"/>
       <c r="M17" s="36"/>
       <c r="N17" s="36"/>
@@ -2480,34 +2510,36 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C18" s="39"/>
       <c r="D18" s="35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E18" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="F18" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="F18" s="35" t="s">
-        <v>38</v>
-      </c>
       <c r="G18" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="I18" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="J18" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="H18" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="I18" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="J18" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="K18" s="36"/>
       <c r="L18" s="36"/>
       <c r="M18" s="36"/>
       <c r="N18" s="36"/>
@@ -2579,17 +2611,17 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C19" s="33"/>
       <c r="D19" s="35" t="n">
         <v>150</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F19" s="35" t="n">
         <v>150</v>
@@ -2606,7 +2638,9 @@
       <c r="J19" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="K19" s="36"/>
+      <c r="K19" s="35" t="n">
+        <v>150</v>
+      </c>
       <c r="L19" s="36"/>
       <c r="M19" s="36"/>
       <c r="N19" s="36"/>
@@ -2678,17 +2712,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="35" t="n">
         <v>55</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F20" s="35" t="n">
         <v>55</v>
@@ -2705,7 +2739,9 @@
       <c r="J20" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="K20" s="36"/>
+      <c r="K20" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="L20" s="36"/>
       <c r="M20" s="36"/>
       <c r="N20" s="36"/>
@@ -2777,17 +2813,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="32" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C21" s="39"/>
       <c r="D21" s="35" t="n">
         <v>72</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F21" s="35" t="n">
         <v>72</v>
@@ -2804,7 +2840,9 @@
       <c r="J21" s="35" t="n">
         <v>72</v>
       </c>
-      <c r="K21" s="36"/>
+      <c r="K21" s="35" t="n">
+        <v>72</v>
+      </c>
       <c r="L21" s="36"/>
       <c r="M21" s="36"/>
       <c r="N21" s="36"/>
@@ -2876,17 +2914,17 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C22" s="39"/>
       <c r="D22" s="35" t="n">
         <v>400</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F22" s="35" t="n">
         <v>400</v>
@@ -2903,7 +2941,9 @@
       <c r="J22" s="35" t="n">
         <v>400</v>
       </c>
-      <c r="K22" s="36"/>
+      <c r="K22" s="35" t="n">
+        <v>400</v>
+      </c>
       <c r="L22" s="36"/>
       <c r="M22" s="36"/>
       <c r="N22" s="36"/>
@@ -2975,34 +3015,36 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B23" s="32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C23" s="33"/>
       <c r="D23" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E23" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="35" t="s">
-        <v>55</v>
-      </c>
       <c r="G23" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H23" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I23" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J23" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="K23" s="36"/>
+        <v>56</v>
+      </c>
+      <c r="K23" s="35" t="s">
+        <v>56</v>
+      </c>
       <c r="L23" s="36"/>
       <c r="M23" s="36"/>
       <c r="N23" s="36"/>
@@ -3074,34 +3116,36 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B24" s="32" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C24" s="33"/>
       <c r="D24" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E24" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="F24" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="35" t="s">
-        <v>59</v>
-      </c>
       <c r="G24" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H24" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I24" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J24" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="K24" s="36"/>
+        <v>60</v>
+      </c>
+      <c r="K24" s="35" t="s">
+        <v>60</v>
+      </c>
       <c r="L24" s="36"/>
       <c r="M24" s="36"/>
       <c r="N24" s="36"/>
@@ -3173,17 +3217,17 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B25" s="32" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F25" s="35" t="n">
         <v>1</v>
@@ -3200,7 +3244,9 @@
       <c r="J25" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K25" s="36"/>
+      <c r="K25" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L25" s="36"/>
       <c r="M25" s="36"/>
       <c r="N25" s="36"/>
@@ -3272,17 +3318,17 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B26" s="32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F26" s="35" t="n">
         <v>1</v>
@@ -3299,7 +3345,9 @@
       <c r="J26" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K26" s="36"/>
+      <c r="K26" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
       <c r="N26" s="36"/>
@@ -3371,17 +3419,17 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C27" s="33"/>
       <c r="D27" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F27" s="35" t="n">
         <v>1</v>
@@ -3398,7 +3446,9 @@
       <c r="J27" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K27" s="36"/>
+      <c r="K27" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L27" s="36"/>
       <c r="M27" s="36"/>
       <c r="N27" s="36"/>
@@ -3470,17 +3520,17 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C28" s="33"/>
       <c r="D28" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F28" s="35" t="n">
         <v>1</v>
@@ -3497,7 +3547,9 @@
       <c r="J28" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K28" s="36"/>
+      <c r="K28" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L28" s="36"/>
       <c r="M28" s="36"/>
       <c r="N28" s="36"/>
@@ -3569,34 +3621,36 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B29" s="32" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C29" s="39"/>
       <c r="D29" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F29" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G29" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H29" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I29" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J29" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="K29" s="36"/>
+        <v>76</v>
+      </c>
+      <c r="K29" s="35" t="s">
+        <v>76</v>
+      </c>
       <c r="L29" s="36"/>
       <c r="M29" s="36"/>
       <c r="N29" s="36"/>
@@ -3668,10 +3722,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B30" s="32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="35" t="n">
@@ -3681,21 +3735,23 @@
         <v>55</v>
       </c>
       <c r="F30" s="35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G30" s="35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H30" s="35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I30" s="35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J30" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="K30" s="36"/>
+        <v>79</v>
+      </c>
+      <c r="K30" s="35" t="s">
+        <v>79</v>
+      </c>
       <c r="L30" s="36"/>
       <c r="M30" s="36"/>
       <c r="N30" s="36"/>
@@ -3767,10 +3823,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B31" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="35" t="n">
@@ -3794,7 +3850,9 @@
       <c r="J31" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="K31" s="36"/>
+      <c r="K31" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
       <c r="N31" s="36"/>
@@ -3866,34 +3924,36 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B32" s="32" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C32" s="33"/>
       <c r="D32" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F32" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G32" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H32" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I32" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J32" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="K32" s="36"/>
+        <v>76</v>
+      </c>
+      <c r="K32" s="35" t="s">
+        <v>76</v>
+      </c>
       <c r="L32" s="36"/>
       <c r="M32" s="36"/>
       <c r="N32" s="36"/>
@@ -3965,34 +4025,36 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B33" s="32" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C33" s="39"/>
       <c r="D33" s="35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F33" s="35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G33" s="35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H33" s="35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I33" s="35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J33" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="K33" s="36"/>
+        <v>86</v>
+      </c>
+      <c r="K33" s="35" t="s">
+        <v>86</v>
+      </c>
       <c r="L33" s="36"/>
       <c r="M33" s="36"/>
       <c r="N33" s="36"/>
@@ -4064,10 +4126,10 @@
     </row>
     <row r="34" s="42" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="40" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B34" s="40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C34" s="16"/>
       <c r="D34" s="41"/>
@@ -4077,6 +4139,7 @@
       <c r="H34" s="41"/>
       <c r="I34" s="41"/>
       <c r="J34" s="41"/>
+      <c r="K34" s="41"/>
       <c r="V34" s="43"/>
       <c r="W34" s="44"/>
       <c r="AN34" s="43"/>
@@ -4088,34 +4151,36 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C35" s="33"/>
       <c r="D35" s="34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E35" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F35" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G35" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I35" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J35" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="K35" s="45"/>
+        <v>92</v>
+      </c>
+      <c r="K35" s="34" t="s">
+        <v>92</v>
+      </c>
       <c r="L35" s="45"/>
       <c r="M35" s="45"/>
       <c r="N35" s="45"/>
@@ -4190,25 +4255,27 @@
         <v>2</v>
       </c>
       <c r="B36" s="48" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C36" s="39"/>
       <c r="D36" s="34"/>
       <c r="E36" s="34"/>
       <c r="F36" s="34"/>
       <c r="G36" s="34" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J36" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="K36" s="36"/>
+        <v>94</v>
+      </c>
+      <c r="K36" s="34" t="s">
+        <v>95</v>
+      </c>
       <c r="L36" s="36"/>
       <c r="M36" s="36"/>
       <c r="N36" s="36"/>
@@ -4280,28 +4347,30 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="48" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B37" s="48" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="34"/>
       <c r="E37" s="34"/>
       <c r="F37" s="34"/>
       <c r="G37" s="34" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H37" s="34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I37" s="34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J37" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="K37" s="36"/>
+        <v>95</v>
+      </c>
+      <c r="K37" s="34" t="s">
+        <v>100</v>
+      </c>
       <c r="L37" s="36"/>
       <c r="M37" s="36"/>
       <c r="N37" s="36"/>
@@ -4373,13 +4442,13 @@
     </row>
     <row r="38" s="42" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="40" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B38" s="40" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D38" s="41"/>
       <c r="E38" s="41"/>
@@ -4388,6 +4457,7 @@
       <c r="H38" s="41"/>
       <c r="I38" s="41"/>
       <c r="J38" s="41"/>
+      <c r="K38" s="41"/>
       <c r="V38" s="43"/>
       <c r="W38" s="44"/>
       <c r="AN38" s="43"/>
@@ -4399,16 +4469,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B39" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C39" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E39" s="34" t="n">
         <v>70</v>
@@ -4428,7 +4498,9 @@
       <c r="J39" s="35" t="n">
         <v>70</v>
       </c>
-      <c r="K39" s="36"/>
+      <c r="K39" s="35" t="n">
+        <v>70</v>
+      </c>
       <c r="L39" s="36"/>
       <c r="M39" s="36"/>
       <c r="N39" s="36"/>
@@ -4500,16 +4572,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B40" s="32" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C40" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E40" s="34" t="n">
         <v>75</v>
@@ -4529,7 +4601,9 @@
       <c r="J40" s="35" t="n">
         <v>75</v>
       </c>
-      <c r="K40" s="36"/>
+      <c r="K40" s="35" t="n">
+        <v>75</v>
+      </c>
       <c r="L40" s="36"/>
       <c r="M40" s="36"/>
       <c r="N40" s="36"/>
@@ -4601,16 +4675,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C41" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E41" s="34" t="n">
         <v>60</v>
@@ -4630,7 +4704,9 @@
       <c r="J41" s="35" t="n">
         <v>60</v>
       </c>
-      <c r="K41" s="36"/>
+      <c r="K41" s="35" t="n">
+        <v>60</v>
+      </c>
       <c r="L41" s="36"/>
       <c r="M41" s="36"/>
       <c r="N41" s="36"/>
@@ -4702,16 +4778,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C42" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E42" s="34" t="n">
         <v>90</v>
@@ -4731,7 +4807,9 @@
       <c r="J42" s="35" t="n">
         <v>90</v>
       </c>
-      <c r="K42" s="36"/>
+      <c r="K42" s="35" t="n">
+        <v>90</v>
+      </c>
       <c r="L42" s="36"/>
       <c r="M42" s="36"/>
       <c r="N42" s="36"/>
@@ -4803,16 +4881,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B43" s="32" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C43" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E43" s="34" t="n">
         <v>1000</v>
@@ -4832,7 +4910,9 @@
       <c r="J43" s="35" t="n">
         <v>1000</v>
       </c>
-      <c r="K43" s="36"/>
+      <c r="K43" s="35" t="n">
+        <v>1000</v>
+      </c>
       <c r="L43" s="36"/>
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
@@ -4904,16 +4984,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C44" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E44" s="34" t="n">
         <v>75</v>
@@ -4933,7 +5013,9 @@
       <c r="J44" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="K44" s="36"/>
+      <c r="K44" s="35" t="n">
+        <v>500</v>
+      </c>
       <c r="L44" s="36"/>
       <c r="M44" s="36"/>
       <c r="N44" s="36"/>
@@ -5005,16 +5087,16 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C45" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E45" s="34" t="n">
         <v>100</v>
@@ -5034,7 +5116,9 @@
       <c r="J45" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="K45" s="36"/>
+      <c r="K45" s="35" t="n">
+        <v>100</v>
+      </c>
       <c r="L45" s="36"/>
       <c r="M45" s="36"/>
       <c r="N45" s="36"/>
@@ -5106,16 +5190,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B46" s="32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C46" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E46" s="34" t="n">
         <v>72</v>
@@ -5135,7 +5219,9 @@
       <c r="J46" s="35" t="n">
         <v>200</v>
       </c>
-      <c r="K46" s="36"/>
+      <c r="K46" s="35" t="n">
+        <v>200</v>
+      </c>
       <c r="L46" s="36"/>
       <c r="M46" s="36"/>
       <c r="N46" s="36"/>
@@ -5207,16 +5293,16 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B47" s="32" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C47" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E47" s="34" t="n">
         <v>65</v>
@@ -5236,7 +5322,9 @@
       <c r="J47" s="35" t="n">
         <v>120</v>
       </c>
-      <c r="K47" s="36"/>
+      <c r="K47" s="35" t="n">
+        <v>120</v>
+      </c>
       <c r="L47" s="36"/>
       <c r="M47" s="36"/>
       <c r="N47" s="36"/>
@@ -5308,16 +5396,16 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B48" s="32" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C48" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E48" s="34" t="n">
         <v>68</v>
@@ -5337,7 +5425,9 @@
       <c r="J48" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="K48" s="36"/>
+      <c r="K48" s="35" t="n">
+        <v>20</v>
+      </c>
       <c r="L48" s="36"/>
       <c r="M48" s="36"/>
       <c r="N48" s="36"/>
@@ -5409,16 +5499,16 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B49" s="32" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C49" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E49" s="34" t="n">
         <v>72</v>
@@ -5438,7 +5528,9 @@
       <c r="J49" s="35" t="n">
         <v>70</v>
       </c>
-      <c r="K49" s="36"/>
+      <c r="K49" s="35" t="n">
+        <v>70</v>
+      </c>
       <c r="L49" s="36"/>
       <c r="M49" s="36"/>
       <c r="N49" s="36"/>
@@ -5510,16 +5602,16 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B50" s="32" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C50" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E50" s="34" t="n">
         <v>72</v>
@@ -5539,7 +5631,9 @@
       <c r="J50" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="K50" s="36"/>
+      <c r="K50" s="35" t="n">
+        <v>150</v>
+      </c>
       <c r="L50" s="36"/>
       <c r="M50" s="36"/>
       <c r="N50" s="36"/>
@@ -5611,19 +5705,19 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B51" s="32" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C51" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E51" s="34" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F51" s="35" t="n">
         <v>55</v>
@@ -5640,7 +5734,9 @@
       <c r="J51" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="K51" s="36"/>
+      <c r="K51" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="L51" s="36"/>
       <c r="M51" s="36"/>
       <c r="N51" s="36"/>
@@ -5712,19 +5808,19 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B52" s="32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C52" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E52" s="34" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F52" s="35" t="n">
         <v>72</v>
@@ -5741,7 +5837,9 @@
       <c r="J52" s="35" t="n">
         <v>72</v>
       </c>
-      <c r="K52" s="36"/>
+      <c r="K52" s="35" t="n">
+        <v>72</v>
+      </c>
       <c r="L52" s="36"/>
       <c r="M52" s="36"/>
       <c r="N52" s="36"/>
@@ -5813,19 +5911,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B53" s="32" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C53" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E53" s="34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F53" s="35" t="n">
         <v>400</v>
@@ -5842,7 +5940,9 @@
       <c r="J53" s="35" t="n">
         <v>400</v>
       </c>
-      <c r="K53" s="36"/>
+      <c r="K53" s="35" t="n">
+        <v>400</v>
+      </c>
       <c r="L53" s="36"/>
       <c r="M53" s="36"/>
       <c r="N53" s="36"/>
@@ -5914,36 +6014,38 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B54" s="32" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C54" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E54" s="34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F54" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G54" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H54" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I54" s="35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J54" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="K54" s="36"/>
+        <v>56</v>
+      </c>
+      <c r="K54" s="35" t="s">
+        <v>56</v>
+      </c>
       <c r="L54" s="36"/>
       <c r="M54" s="36"/>
       <c r="N54" s="36"/>
@@ -6015,36 +6117,38 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="32" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B55" s="32" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C55" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E55" s="34" t="n">
         <v>72</v>
       </c>
       <c r="F55" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G55" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H55" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I55" s="35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J55" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="K55" s="36"/>
+        <v>60</v>
+      </c>
+      <c r="K55" s="35" t="s">
+        <v>60</v>
+      </c>
       <c r="L55" s="36"/>
       <c r="M55" s="36"/>
       <c r="N55" s="36"/>
@@ -6116,16 +6220,16 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="32" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B56" s="32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C56" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E56" s="34" t="n">
         <v>720</v>
@@ -6145,7 +6249,9 @@
       <c r="J56" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K56" s="36"/>
+      <c r="K56" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L56" s="36"/>
       <c r="M56" s="36"/>
       <c r="N56" s="36"/>
@@ -6217,16 +6323,16 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="32" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B57" s="32" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C57" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E57" s="34" t="n">
         <v>48</v>
@@ -6246,7 +6352,9 @@
       <c r="J57" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K57" s="36"/>
+      <c r="K57" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L57" s="36"/>
       <c r="M57" s="36"/>
       <c r="N57" s="36"/>
@@ -6318,16 +6426,16 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="32" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B58" s="32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C58" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E58" s="34" t="n">
         <v>72</v>
@@ -6347,7 +6455,9 @@
       <c r="J58" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K58" s="36"/>
+      <c r="K58" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L58" s="36"/>
       <c r="M58" s="36"/>
       <c r="N58" s="36"/>
@@ -6419,16 +6529,16 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B59" s="32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C59" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D59" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E59" s="34" t="n">
         <v>84</v>
@@ -6448,7 +6558,9 @@
       <c r="J59" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="K59" s="36"/>
+      <c r="K59" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="L59" s="36"/>
       <c r="M59" s="36"/>
       <c r="N59" s="36"/>
@@ -6520,19 +6632,19 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="32" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B60" s="32" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C60" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D60" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E60" s="34" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F60" s="35" t="n">
         <v>55</v>
@@ -6549,7 +6661,9 @@
       <c r="J60" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="K60" s="36"/>
+      <c r="K60" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="L60" s="36"/>
       <c r="M60" s="36"/>
       <c r="N60" s="36"/>
@@ -6621,19 +6735,19 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B61" s="32" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C61" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E61" s="34" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F61" s="35" t="n">
         <v>55</v>
@@ -6650,7 +6764,9 @@
       <c r="J61" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="K61" s="36"/>
+      <c r="K61" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="L61" s="36"/>
       <c r="M61" s="36"/>
       <c r="N61" s="36"/>
@@ -6721,9 +6837,9 @@
       <c r="CA61" s="36"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K8:ZZ33 K39:ZZ61">
+  <conditionalFormatting sqref="L8:ZZ33 L39:ZZ61">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>#ref!&lt;&gt;K8</formula>
+      <formula>#ref!&lt;&gt;L8</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Add step to footest for expected value =LAST with tolerance
</commit_message>
<xml_diff>
--- a/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
+++ b/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="132">
   <si>
     <t xml:space="preserve">Dummy Test</t>
   </si>
@@ -206,6 +206,9 @@
     <t xml:space="preserve">8</t>
   </si>
   <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
     <t xml:space="preserve">A</t>
   </si>
   <si>
@@ -411,6 +414,9 @@
   </si>
   <si>
     <t xml:space="preserve">ts_u24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">55.04</t>
   </si>
   <si>
     <t xml:space="preserve">Y</t>
@@ -1324,7 +1330,9 @@
       <c r="K6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="L6" s="19"/>
+      <c r="L6" s="18" t="s">
+        <v>4</v>
+      </c>
       <c r="M6" s="19"/>
       <c r="N6" s="19"/>
       <c r="O6" s="19"/>
@@ -1429,7 +1437,9 @@
       <c r="K7" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="26"/>
+      <c r="L7" s="25" t="s">
+        <v>13</v>
+      </c>
       <c r="M7" s="26"/>
       <c r="N7" s="26"/>
       <c r="O7" s="26"/>
@@ -1500,10 +1510,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="32" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" s="33"/>
       <c r="D8" s="34" t="n">
@@ -1530,7 +1540,9 @@
       <c r="K8" s="35" t="n">
         <v>70</v>
       </c>
-      <c r="L8" s="36"/>
+      <c r="L8" s="35" t="n">
+        <v>70</v>
+      </c>
       <c r="M8" s="36"/>
       <c r="N8" s="36"/>
       <c r="O8" s="36"/>
@@ -1601,10 +1613,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="33"/>
       <c r="D9" s="35" t="n">
@@ -1631,7 +1643,9 @@
       <c r="K9" s="35" t="n">
         <v>75</v>
       </c>
-      <c r="L9" s="36"/>
+      <c r="L9" s="35" t="n">
+        <v>75</v>
+      </c>
       <c r="M9" s="36"/>
       <c r="N9" s="36"/>
       <c r="O9" s="36"/>
@@ -1702,10 +1716,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="39"/>
       <c r="D10" s="35" t="n">
@@ -1732,7 +1746,9 @@
       <c r="K10" s="35" t="n">
         <v>60</v>
       </c>
-      <c r="L10" s="36"/>
+      <c r="L10" s="35" t="n">
+        <v>60</v>
+      </c>
       <c r="M10" s="36"/>
       <c r="N10" s="36"/>
       <c r="O10" s="36"/>
@@ -1803,10 +1819,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" s="39"/>
       <c r="D11" s="35" t="n">
@@ -1833,7 +1849,9 @@
       <c r="K11" s="35" t="n">
         <v>90</v>
       </c>
-      <c r="L11" s="36"/>
+      <c r="L11" s="35" t="n">
+        <v>90</v>
+      </c>
       <c r="M11" s="36"/>
       <c r="N11" s="36"/>
       <c r="O11" s="36"/>
@@ -1904,10 +1922,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C12" s="33"/>
       <c r="D12" s="35" t="n">
@@ -1934,7 +1952,9 @@
       <c r="K12" s="35" t="n">
         <v>1000</v>
       </c>
-      <c r="L12" s="36"/>
+      <c r="L12" s="35" t="n">
+        <v>1000</v>
+      </c>
       <c r="M12" s="36"/>
       <c r="N12" s="36"/>
       <c r="O12" s="36"/>
@@ -2005,17 +2025,17 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C13" s="39"/>
       <c r="D13" s="35" t="n">
         <v>500</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F13" s="35" t="n">
         <v>500</v>
@@ -2035,7 +2055,9 @@
       <c r="K13" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="L13" s="36"/>
+      <c r="L13" s="35" t="n">
+        <v>500</v>
+      </c>
       <c r="M13" s="36"/>
       <c r="N13" s="36"/>
       <c r="O13" s="36"/>
@@ -2106,10 +2128,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14" s="32" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C14" s="39"/>
       <c r="D14" s="35" t="n">
@@ -2136,7 +2158,9 @@
       <c r="K14" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="L14" s="36"/>
+      <c r="L14" s="35" t="n">
+        <v>100</v>
+      </c>
       <c r="M14" s="36"/>
       <c r="N14" s="36"/>
       <c r="O14" s="36"/>
@@ -2207,17 +2231,17 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="35" t="n">
         <v>200</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F15" s="35" t="n">
         <v>200</v>
@@ -2237,7 +2261,9 @@
       <c r="K15" s="35" t="n">
         <v>200</v>
       </c>
-      <c r="L15" s="36"/>
+      <c r="L15" s="35" t="n">
+        <v>200</v>
+      </c>
       <c r="M15" s="36"/>
       <c r="N15" s="36"/>
       <c r="O15" s="36"/>
@@ -2308,17 +2334,17 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="32" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="35" t="n">
         <v>120</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F16" s="35" t="n">
         <v>120</v>
@@ -2338,7 +2364,9 @@
       <c r="K16" s="35" t="n">
         <v>120</v>
       </c>
-      <c r="L16" s="36"/>
+      <c r="L16" s="35" t="n">
+        <v>120</v>
+      </c>
       <c r="M16" s="36"/>
       <c r="N16" s="36"/>
       <c r="O16" s="36"/>
@@ -2409,17 +2437,17 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B17" s="32" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C17" s="33"/>
       <c r="D17" s="35" t="n">
         <v>20</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F17" s="35" t="n">
         <v>20</v>
@@ -2439,7 +2467,9 @@
       <c r="K17" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="L17" s="36"/>
+      <c r="L17" s="35" t="n">
+        <v>20</v>
+      </c>
       <c r="M17" s="36"/>
       <c r="N17" s="36"/>
       <c r="O17" s="36"/>
@@ -2510,37 +2540,39 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="32" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18" s="39"/>
       <c r="D18" s="35" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E18" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="35" t="s">
-        <v>39</v>
-      </c>
       <c r="G18" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="J18" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="K18" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H18" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="I18" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="J18" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="K18" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="L18" s="36"/>
+      <c r="L18" s="35" t="s">
+        <v>42</v>
+      </c>
       <c r="M18" s="36"/>
       <c r="N18" s="36"/>
       <c r="O18" s="36"/>
@@ -2611,17 +2643,17 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C19" s="33"/>
       <c r="D19" s="35" t="n">
         <v>150</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F19" s="35" t="n">
         <v>150</v>
@@ -2641,7 +2673,9 @@
       <c r="K19" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="L19" s="36"/>
+      <c r="L19" s="35" t="n">
+        <v>150</v>
+      </c>
       <c r="M19" s="36"/>
       <c r="N19" s="36"/>
       <c r="O19" s="36"/>
@@ -2712,17 +2746,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="35" t="n">
         <v>55</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F20" s="35" t="n">
         <v>55</v>
@@ -2742,7 +2776,9 @@
       <c r="K20" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="L20" s="36"/>
+      <c r="L20" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="M20" s="36"/>
       <c r="N20" s="36"/>
       <c r="O20" s="36"/>
@@ -2813,17 +2849,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" s="32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C21" s="39"/>
       <c r="D21" s="35" t="n">
         <v>72</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F21" s="35" t="n">
         <v>72</v>
@@ -2843,7 +2879,9 @@
       <c r="K21" s="35" t="n">
         <v>72</v>
       </c>
-      <c r="L21" s="36"/>
+      <c r="L21" s="35" t="n">
+        <v>72</v>
+      </c>
       <c r="M21" s="36"/>
       <c r="N21" s="36"/>
       <c r="O21" s="36"/>
@@ -2914,17 +2952,17 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B22" s="32" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C22" s="39"/>
       <c r="D22" s="35" t="n">
         <v>400</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F22" s="35" t="n">
         <v>400</v>
@@ -2944,7 +2982,9 @@
       <c r="K22" s="35" t="n">
         <v>400</v>
       </c>
-      <c r="L22" s="36"/>
+      <c r="L22" s="35" t="n">
+        <v>400</v>
+      </c>
       <c r="M22" s="36"/>
       <c r="N22" s="36"/>
       <c r="O22" s="36"/>
@@ -3015,37 +3055,39 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B23" s="32" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C23" s="33"/>
       <c r="D23" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E23" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="F23" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="F23" s="35" t="s">
-        <v>56</v>
-      </c>
       <c r="G23" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H23" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I23" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J23" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K23" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="L23" s="36"/>
+        <v>57</v>
+      </c>
+      <c r="L23" s="35" t="s">
+        <v>57</v>
+      </c>
       <c r="M23" s="36"/>
       <c r="N23" s="36"/>
       <c r="O23" s="36"/>
@@ -3116,37 +3158,39 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B24" s="32" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C24" s="33"/>
       <c r="D24" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E24" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="F24" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="35" t="s">
-        <v>60</v>
-      </c>
       <c r="G24" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H24" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I24" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J24" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K24" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="L24" s="36"/>
+        <v>61</v>
+      </c>
+      <c r="L24" s="35" t="s">
+        <v>61</v>
+      </c>
       <c r="M24" s="36"/>
       <c r="N24" s="36"/>
       <c r="O24" s="36"/>
@@ -3217,17 +3261,17 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B25" s="32" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F25" s="35" t="n">
         <v>1</v>
@@ -3247,7 +3291,9 @@
       <c r="K25" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L25" s="36"/>
+      <c r="L25" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M25" s="36"/>
       <c r="N25" s="36"/>
       <c r="O25" s="36"/>
@@ -3318,17 +3364,17 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B26" s="32" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F26" s="35" t="n">
         <v>1</v>
@@ -3348,7 +3394,9 @@
       <c r="K26" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L26" s="36"/>
+      <c r="L26" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M26" s="36"/>
       <c r="N26" s="36"/>
       <c r="O26" s="36"/>
@@ -3419,17 +3467,17 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C27" s="33"/>
       <c r="D27" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F27" s="35" t="n">
         <v>1</v>
@@ -3449,7 +3497,9 @@
       <c r="K27" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L27" s="36"/>
+      <c r="L27" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M27" s="36"/>
       <c r="N27" s="36"/>
       <c r="O27" s="36"/>
@@ -3520,17 +3570,17 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C28" s="33"/>
       <c r="D28" s="35" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F28" s="35" t="n">
         <v>1</v>
@@ -3550,7 +3600,9 @@
       <c r="K28" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L28" s="36"/>
+      <c r="L28" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M28" s="36"/>
       <c r="N28" s="36"/>
       <c r="O28" s="36"/>
@@ -3621,37 +3673,39 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B29" s="32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C29" s="39"/>
       <c r="D29" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F29" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G29" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H29" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I29" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J29" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K29" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="L29" s="36"/>
+        <v>77</v>
+      </c>
+      <c r="L29" s="35" t="s">
+        <v>77</v>
+      </c>
       <c r="M29" s="36"/>
       <c r="N29" s="36"/>
       <c r="O29" s="36"/>
@@ -3722,10 +3776,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B30" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="35" t="n">
@@ -3735,24 +3789,26 @@
         <v>55</v>
       </c>
       <c r="F30" s="35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G30" s="35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H30" s="35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I30" s="35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J30" s="35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K30" s="35" t="s">
-        <v>79</v>
-      </c>
-      <c r="L30" s="36"/>
+        <v>80</v>
+      </c>
+      <c r="L30" s="35" t="s">
+        <v>80</v>
+      </c>
       <c r="M30" s="36"/>
       <c r="N30" s="36"/>
       <c r="O30" s="36"/>
@@ -3823,10 +3879,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B31" s="32" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="35" t="n">
@@ -3853,7 +3909,9 @@
       <c r="K31" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="L31" s="36"/>
+      <c r="L31" s="35" t="s">
+        <v>83</v>
+      </c>
       <c r="M31" s="36"/>
       <c r="N31" s="36"/>
       <c r="O31" s="36"/>
@@ -3924,37 +3982,39 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="32" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C32" s="33"/>
       <c r="D32" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F32" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G32" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H32" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I32" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J32" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K32" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="L32" s="36"/>
+        <v>77</v>
+      </c>
+      <c r="L32" s="35" t="s">
+        <v>77</v>
+      </c>
       <c r="M32" s="36"/>
       <c r="N32" s="36"/>
       <c r="O32" s="36"/>
@@ -4025,37 +4085,39 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B33" s="32" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C33" s="39"/>
       <c r="D33" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F33" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G33" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H33" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I33" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="J33" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K33" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="L33" s="36"/>
+        <v>88</v>
+      </c>
+      <c r="L33" s="35" t="s">
+        <v>88</v>
+      </c>
       <c r="M33" s="36"/>
       <c r="N33" s="36"/>
       <c r="O33" s="36"/>
@@ -4126,10 +4188,10 @@
     </row>
     <row r="34" s="42" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="40" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B34" s="40" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C34" s="16"/>
       <c r="D34" s="41"/>
@@ -4140,6 +4202,7 @@
       <c r="I34" s="41"/>
       <c r="J34" s="41"/>
       <c r="K34" s="41"/>
+      <c r="L34" s="41"/>
       <c r="V34" s="43"/>
       <c r="W34" s="44"/>
       <c r="AN34" s="43"/>
@@ -4151,37 +4214,39 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C35" s="33"/>
       <c r="D35" s="34" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E35" s="34" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F35" s="34" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G35" s="34" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I35" s="34" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="J35" s="34" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K35" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="L35" s="45"/>
+        <v>94</v>
+      </c>
+      <c r="L35" s="34" t="s">
+        <v>93</v>
+      </c>
       <c r="M35" s="45"/>
       <c r="N35" s="45"/>
       <c r="O35" s="45"/>
@@ -4255,28 +4320,28 @@
         <v>2</v>
       </c>
       <c r="B36" s="48" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C36" s="39"/>
       <c r="D36" s="34"/>
       <c r="E36" s="34"/>
       <c r="F36" s="34"/>
       <c r="G36" s="34" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J36" s="34" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K36" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="L36" s="36"/>
+        <v>97</v>
+      </c>
+      <c r="L36" s="34"/>
       <c r="M36" s="36"/>
       <c r="N36" s="36"/>
       <c r="O36" s="36"/>
@@ -4347,31 +4412,31 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="48" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B37" s="48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="34"/>
       <c r="E37" s="34"/>
       <c r="F37" s="34"/>
       <c r="G37" s="34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H37" s="34" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I37" s="34" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J37" s="34" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K37" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="L37" s="36"/>
+        <v>102</v>
+      </c>
+      <c r="L37" s="34"/>
       <c r="M37" s="36"/>
       <c r="N37" s="36"/>
       <c r="O37" s="36"/>
@@ -4442,13 +4507,13 @@
     </row>
     <row r="38" s="42" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="40" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B38" s="40" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D38" s="41"/>
       <c r="E38" s="41"/>
@@ -4458,6 +4523,7 @@
       <c r="I38" s="41"/>
       <c r="J38" s="41"/>
       <c r="K38" s="41"/>
+      <c r="L38" s="41"/>
       <c r="V38" s="43"/>
       <c r="W38" s="44"/>
       <c r="AN38" s="43"/>
@@ -4469,16 +4535,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B39" s="32" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C39" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E39" s="34" t="n">
         <v>70</v>
@@ -4501,7 +4567,9 @@
       <c r="K39" s="35" t="n">
         <v>70</v>
       </c>
-      <c r="L39" s="36"/>
+      <c r="L39" s="35" t="n">
+        <v>70</v>
+      </c>
       <c r="M39" s="36"/>
       <c r="N39" s="36"/>
       <c r="O39" s="36"/>
@@ -4572,16 +4640,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B40" s="32" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C40" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E40" s="34" t="n">
         <v>75</v>
@@ -4604,7 +4672,9 @@
       <c r="K40" s="35" t="n">
         <v>75</v>
       </c>
-      <c r="L40" s="36"/>
+      <c r="L40" s="35" t="n">
+        <v>75</v>
+      </c>
       <c r="M40" s="36"/>
       <c r="N40" s="36"/>
       <c r="O40" s="36"/>
@@ -4675,16 +4745,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C41" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E41" s="34" t="n">
         <v>60</v>
@@ -4707,7 +4777,9 @@
       <c r="K41" s="35" t="n">
         <v>60</v>
       </c>
-      <c r="L41" s="36"/>
+      <c r="L41" s="35" t="n">
+        <v>60</v>
+      </c>
       <c r="M41" s="36"/>
       <c r="N41" s="36"/>
       <c r="O41" s="36"/>
@@ -4778,16 +4850,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C42" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E42" s="34" t="n">
         <v>90</v>
@@ -4810,7 +4882,9 @@
       <c r="K42" s="35" t="n">
         <v>90</v>
       </c>
-      <c r="L42" s="36"/>
+      <c r="L42" s="35" t="n">
+        <v>90</v>
+      </c>
       <c r="M42" s="36"/>
       <c r="N42" s="36"/>
       <c r="O42" s="36"/>
@@ -4881,16 +4955,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B43" s="32" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C43" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E43" s="34" t="n">
         <v>1000</v>
@@ -4913,7 +4987,9 @@
       <c r="K43" s="35" t="n">
         <v>1000</v>
       </c>
-      <c r="L43" s="36"/>
+      <c r="L43" s="35" t="n">
+        <v>1000</v>
+      </c>
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
       <c r="O43" s="36"/>
@@ -4984,16 +5060,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C44" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E44" s="34" t="n">
         <v>75</v>
@@ -5016,7 +5092,9 @@
       <c r="K44" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="L44" s="36"/>
+      <c r="L44" s="35" t="n">
+        <v>500</v>
+      </c>
       <c r="M44" s="36"/>
       <c r="N44" s="36"/>
       <c r="O44" s="36"/>
@@ -5087,16 +5165,16 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C45" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E45" s="34" t="n">
         <v>100</v>
@@ -5119,7 +5197,9 @@
       <c r="K45" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="L45" s="36"/>
+      <c r="L45" s="35" t="n">
+        <v>100</v>
+      </c>
       <c r="M45" s="36"/>
       <c r="N45" s="36"/>
       <c r="O45" s="36"/>
@@ -5190,16 +5270,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B46" s="32" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C46" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E46" s="34" t="n">
         <v>72</v>
@@ -5222,7 +5302,9 @@
       <c r="K46" s="35" t="n">
         <v>200</v>
       </c>
-      <c r="L46" s="36"/>
+      <c r="L46" s="35" t="n">
+        <v>200</v>
+      </c>
       <c r="M46" s="36"/>
       <c r="N46" s="36"/>
       <c r="O46" s="36"/>
@@ -5293,16 +5375,16 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B47" s="32" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C47" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E47" s="34" t="n">
         <v>65</v>
@@ -5325,7 +5407,9 @@
       <c r="K47" s="35" t="n">
         <v>120</v>
       </c>
-      <c r="L47" s="36"/>
+      <c r="L47" s="35" t="n">
+        <v>120</v>
+      </c>
       <c r="M47" s="36"/>
       <c r="N47" s="36"/>
       <c r="O47" s="36"/>
@@ -5396,16 +5480,16 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B48" s="32" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C48" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E48" s="34" t="n">
         <v>68</v>
@@ -5428,7 +5512,9 @@
       <c r="K48" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="L48" s="36"/>
+      <c r="L48" s="35" t="n">
+        <v>20</v>
+      </c>
       <c r="M48" s="36"/>
       <c r="N48" s="36"/>
       <c r="O48" s="36"/>
@@ -5499,16 +5585,16 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B49" s="32" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C49" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E49" s="34" t="n">
         <v>72</v>
@@ -5531,7 +5617,9 @@
       <c r="K49" s="35" t="n">
         <v>70</v>
       </c>
-      <c r="L49" s="36"/>
+      <c r="L49" s="35" t="n">
+        <v>70</v>
+      </c>
       <c r="M49" s="36"/>
       <c r="N49" s="36"/>
       <c r="O49" s="36"/>
@@ -5602,16 +5690,16 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B50" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C50" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E50" s="34" t="n">
         <v>72</v>
@@ -5634,7 +5722,9 @@
       <c r="K50" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="L50" s="36"/>
+      <c r="L50" s="35" t="n">
+        <v>150</v>
+      </c>
       <c r="M50" s="36"/>
       <c r="N50" s="36"/>
       <c r="O50" s="36"/>
@@ -5705,19 +5795,19 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B51" s="32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C51" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E51" s="34" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F51" s="35" t="n">
         <v>55</v>
@@ -5737,7 +5827,9 @@
       <c r="K51" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="L51" s="36"/>
+      <c r="L51" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="M51" s="36"/>
       <c r="N51" s="36"/>
       <c r="O51" s="36"/>
@@ -5808,19 +5900,19 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B52" s="32" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C52" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E52" s="34" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F52" s="35" t="n">
         <v>72</v>
@@ -5840,7 +5932,9 @@
       <c r="K52" s="35" t="n">
         <v>72</v>
       </c>
-      <c r="L52" s="36"/>
+      <c r="L52" s="35" t="n">
+        <v>72</v>
+      </c>
       <c r="M52" s="36"/>
       <c r="N52" s="36"/>
       <c r="O52" s="36"/>
@@ -5911,19 +6005,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B53" s="32" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C53" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E53" s="34" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F53" s="35" t="n">
         <v>400</v>
@@ -5943,7 +6037,9 @@
       <c r="K53" s="35" t="n">
         <v>400</v>
       </c>
-      <c r="L53" s="36"/>
+      <c r="L53" s="35" t="n">
+        <v>400</v>
+      </c>
       <c r="M53" s="36"/>
       <c r="N53" s="36"/>
       <c r="O53" s="36"/>
@@ -6014,39 +6110,41 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B54" s="32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C54" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E54" s="34" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F54" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G54" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H54" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I54" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J54" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K54" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="L54" s="36"/>
+        <v>57</v>
+      </c>
+      <c r="L54" s="35" t="s">
+        <v>57</v>
+      </c>
       <c r="M54" s="36"/>
       <c r="N54" s="36"/>
       <c r="O54" s="36"/>
@@ -6117,39 +6215,41 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="32" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B55" s="32" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C55" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E55" s="34" t="n">
         <v>72</v>
       </c>
       <c r="F55" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G55" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H55" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I55" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J55" s="35" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K55" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="L55" s="36"/>
+        <v>61</v>
+      </c>
+      <c r="L55" s="35" t="s">
+        <v>61</v>
+      </c>
       <c r="M55" s="36"/>
       <c r="N55" s="36"/>
       <c r="O55" s="36"/>
@@ -6220,16 +6320,16 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="32" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B56" s="32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C56" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E56" s="34" t="n">
         <v>720</v>
@@ -6252,7 +6352,9 @@
       <c r="K56" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L56" s="36"/>
+      <c r="L56" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M56" s="36"/>
       <c r="N56" s="36"/>
       <c r="O56" s="36"/>
@@ -6323,16 +6425,16 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="32" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B57" s="32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C57" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E57" s="34" t="n">
         <v>48</v>
@@ -6355,7 +6457,9 @@
       <c r="K57" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L57" s="36"/>
+      <c r="L57" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M57" s="36"/>
       <c r="N57" s="36"/>
       <c r="O57" s="36"/>
@@ -6426,16 +6530,16 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B58" s="32" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C58" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E58" s="34" t="n">
         <v>72</v>
@@ -6458,7 +6562,9 @@
       <c r="K58" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L58" s="36"/>
+      <c r="L58" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M58" s="36"/>
       <c r="N58" s="36"/>
       <c r="O58" s="36"/>
@@ -6529,16 +6635,16 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B59" s="32" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C59" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D59" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E59" s="34" t="n">
         <v>84</v>
@@ -6561,7 +6667,9 @@
       <c r="K59" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="L59" s="36"/>
+      <c r="L59" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="M59" s="36"/>
       <c r="N59" s="36"/>
       <c r="O59" s="36"/>
@@ -6632,19 +6740,19 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B60" s="32" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C60" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D60" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E60" s="34" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F60" s="35" t="n">
         <v>55</v>
@@ -6664,7 +6772,9 @@
       <c r="K60" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="L60" s="36"/>
+      <c r="L60" s="35" t="n">
+        <v>55</v>
+      </c>
       <c r="M60" s="36"/>
       <c r="N60" s="36"/>
       <c r="O60" s="36"/>
@@ -6735,19 +6845,19 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B61" s="32" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C61" s="33" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E61" s="34" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F61" s="35" t="n">
         <v>55</v>
@@ -6767,7 +6877,9 @@
       <c r="K61" s="35" t="n">
         <v>55</v>
       </c>
-      <c r="L61" s="36"/>
+      <c r="L61" s="35" t="s">
+        <v>80</v>
+      </c>
       <c r="M61" s="36"/>
       <c r="N61" s="36"/>
       <c r="O61" s="36"/>
@@ -6837,9 +6949,9 @@
       <c r="CA61" s="36"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L8:ZZ33 L39:ZZ61">
+  <conditionalFormatting sqref="M8:ZZ33 M39:ZZ61">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>#ref!&lt;&gt;L8</formula>
+      <formula>#ref!&lt;&gt;M8</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>